<commit_message>
Podvoji projekt, plošče iz slicerja, zaokroževanje ponudbe, statusi Ponudba/Sprejeto/Natisnjeno/Plačano; Excel v6 plošče + zaokroževanje
</commit_message>
<xml_diff>
--- a/excel/HS_3D_Kalkulator_v6.xlsx
+++ b/excel/HS_3D_Kalkulator_v6.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poslovne nastavitve" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datoteke" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projekti" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plošče" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +33,7 @@
     <numFmt numFmtId="170" formatCode="0.0000"/>
     <numFmt numFmtId="171" formatCode="0.00 %"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -114,6 +115,11 @@
     <font>
       <color rgb="00334155"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000284C7"/>
+      <sz val="14"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -169,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -221,6 +227,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -969,7 +978,7 @@
         </is>
       </c>
       <c r="F12" s="14">
-        <f>IF($C$16="DA",$C$17+$C$18/60,$C$12*($C$14+$C$15/60))</f>
+        <f>IF('Plošče'!$B$2="DA",'Plošče'!$B$16,IF($C$16="DA",$C$17+$C$18/60,$C$12*($C$14+$C$15/60)))</f>
         <v/>
       </c>
     </row>
@@ -988,7 +997,7 @@
         </is>
       </c>
       <c r="F13" s="16">
-        <f>($C$12*$C$13+$C$19)/1000</f>
+        <f>(IF('Plošče'!$B$2="DA",'Plošče'!$D$16,$C$12*$C$13)+$C$19)/1000</f>
         <v/>
       </c>
     </row>
@@ -1119,7 +1128,7 @@
         </is>
       </c>
       <c r="F20" s="18">
-        <f>F13*F15</f>
+        <f>IF('Plošče'!$B$2="DA",'Plošče'!$F$16+$C$19/1000*F15,F13*F15)</f>
         <v/>
       </c>
     </row>
@@ -1591,11 +1600,11 @@
     <row r="42">
       <c r="E42" t="inlineStr">
         <is>
-          <t>PRIHODEK brez DDV</t>
+          <t>PRIHODEK brez DDV (zaokroženo navzgor)</t>
         </is>
       </c>
       <c r="F42" s="18">
-        <f>MAX(0,IF(F41,'Cenik storitev'!$B$9,F40))</f>
+        <f>IF(AND(NOT($C$7="Zase"),'Cenik storitev'!$B$16&gt;0,MAX(0,IF(F41,'Cenik storitev'!$B$9,F40))&gt;0),CEILING(ROUND(MAX(0,IF(F41,'Cenik storitev'!$B$9,F40)),2),'Cenik storitev'!$B$16),MAX(0,IF(F41,'Cenik storitev'!$B$9,F40)))</f>
         <v/>
       </c>
       <c r="J42" t="inlineStr">
@@ -3840,7 +3849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -4045,6 +4054,21 @@
         <v>30</v>
       </c>
       <c r="C15" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Zaokroževanje ponudbe navzgor (0 = izklop, 1 ali 5)</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -5145,4 +5169,266 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>Plošče iz slicerja (Bambu Studio / PrusaSlicer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Uporabi plošče (DA/NE)</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Če je DA: čas in grami celega naročila = vsota plošč (število kosov se ne množi). Dodatna poraba (Kalkulator C19) se prišteje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>Plošča</t>
+        </is>
+      </c>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>Ure</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>Minute</t>
+        </is>
+      </c>
+      <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>Grami</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="F4" s="23" t="inlineStr">
+        <is>
+          <t>Strošek materiala</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Plošča 1</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n"/>
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="15" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="26">
+        <f>IF(OR(D5="",E5=""),0,D5/1000*IFERROR(INDEX(Materiali!$H:$H,MATCH(E5,Materiali!$A:$A,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Plošča 2</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n"/>
+      <c r="C6" s="15" t="n"/>
+      <c r="D6" s="15" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="26">
+        <f>IF(OR(D6="",E6=""),0,D6/1000*IFERROR(INDEX(Materiali!$H:$H,MATCH(E6,Materiali!$A:$A,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Plošča 3</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n"/>
+      <c r="C7" s="15" t="n"/>
+      <c r="D7" s="15" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="26">
+        <f>IF(OR(D7="",E7=""),0,D7/1000*IFERROR(INDEX(Materiali!$H:$H,MATCH(E7,Materiali!$A:$A,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Plošča 4</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="15" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="26">
+        <f>IF(OR(D8="",E8=""),0,D8/1000*IFERROR(INDEX(Materiali!$H:$H,MATCH(E8,Materiali!$A:$A,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Plošča 5</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="26">
+        <f>IF(OR(D9="",E9=""),0,D9/1000*IFERROR(INDEX(Materiali!$H:$H,MATCH(E9,Materiali!$A:$A,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Plošča 6</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="26">
+        <f>IF(OR(D10="",E10=""),0,D10/1000*IFERROR(INDEX(Materiali!$H:$H,MATCH(E10,Materiali!$A:$A,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Plošča 7</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="26">
+        <f>IF(OR(D11="",E11=""),0,D11/1000*IFERROR(INDEX(Materiali!$H:$H,MATCH(E11,Materiali!$A:$A,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Plošča 8</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="26">
+        <f>IF(OR(D12="",E12=""),0,D12/1000*IFERROR(INDEX(Materiali!$H:$H,MATCH(E12,Materiali!$A:$A,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Plošča 9</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="26">
+        <f>IF(OR(D13="",E13=""),0,D13/1000*IFERROR(INDEX(Materiali!$H:$H,MATCH(E13,Materiali!$A:$A,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Plošča 10</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="26">
+        <f>IF(OR(D14="",E14=""),0,D14/1000*IFERROR(INDEX(Materiali!$H:$H,MATCH(E14,Materiali!$A:$A,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>SKUPAJ</t>
+        </is>
+      </c>
+      <c r="B16" s="40">
+        <f>SUM(B5:B14)+SUM(C5:C14)/60</f>
+        <v/>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>h skupaj</t>
+        </is>
+      </c>
+      <c r="D16" s="41">
+        <f>SUM(D5:D14)</f>
+        <v/>
+      </c>
+      <c r="F16" s="34">
+        <f>SUM(F5:F14)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"DA,NE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E5 E6 E7 E8 E9 E10 E11 E12 E13 E14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Materiali!$A$4:$A$45</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>